<commit_message>
further dev in rc rover programming
</commit_message>
<xml_diff>
--- a/rc_rover/BOM.xlsx
+++ b/rc_rover/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -49,10 +49,19 @@
     <t xml:space="preserve">STC8H8K64U</t>
   </si>
   <si>
+    <t xml:space="preserve">ALREADY BOUGHT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perf Board</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raspberry Pi Pico</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIP28 socket</t>
   </si>
   <si>
-    <t xml:space="preserve">LM317</t>
+    <t xml:space="preserve">LM338</t>
   </si>
   <si>
     <t xml:space="preserve">L7805</t>
@@ -79,9 +88,6 @@
     <t xml:space="preserve">nRF24l01</t>
   </si>
   <si>
-    <t xml:space="preserve">ALREADY BOUGHT</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pin Header 2x3</t>
   </si>
   <si>
@@ -95,6 +101,9 @@
   </si>
   <si>
     <t xml:space="preserve">including dc motor ones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ultrasonic Mount</t>
   </si>
   <si>
     <t xml:space="preserve">Ultrasonic Sensor</t>
@@ -504,8 +513,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
-  <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G41"/>
+  <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.39"/>
@@ -576,7 +585,9 @@
         <f aca="false">C3*D3</f>
         <v>100</v>
       </c>
-      <c r="F3" s="13"/>
+      <c r="F3" s="0" t="s">
+        <v>9</v>
+      </c>
       <c r="G3" s="12"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -584,19 +595,18 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="12" t="n">
         <f aca="false">C4*D4</f>
-        <v>3</v>
-      </c>
-      <c r="F4" s="13"/>
+        <v>10</v>
+      </c>
       <c r="G4" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -604,17 +614,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="12" t="n">
-        <f aca="false">C5*D5</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="12"/>
@@ -624,17 +633,17 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="12" t="n">
         <f aca="false">C6*D6</f>
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F6" s="13"/>
       <c r="G6" s="12"/>
@@ -644,18 +653,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="12" t="n">
         <f aca="false">C7*D7</f>
-        <v>4</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F7" s="13"/>
       <c r="G7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -663,7 +673,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="11" t="n">
         <v>15</v>
@@ -675,6 +685,7 @@
         <f aca="false">C8*D8</f>
         <v>15</v>
       </c>
+      <c r="F8" s="13"/>
       <c r="G8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -682,13 +693,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">C9*D9</f>
@@ -701,17 +712,17 @@
         <v>9</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="11" t="n">
         <v>15</v>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>5</v>
       </c>
       <c r="D10" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">C10*D10</f>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G10" s="12"/>
     </row>
@@ -720,17 +731,17 @@
         <v>10</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">C11*D11</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" s="12"/>
     </row>
@@ -739,17 +750,17 @@
         <v>11</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>680</v>
+        <v>5</v>
       </c>
       <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="12" t="n">
         <f aca="false">C12*D12</f>
-        <v>680</v>
+        <v>5</v>
       </c>
       <c r="G12" s="12"/>
     </row>
@@ -758,20 +769,17 @@
         <v>12</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D13" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="12" t="n">
         <f aca="false">C13*D13</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="0" t="s">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="G13" s="12"/>
     </row>
@@ -783,14 +791,14 @@
         <v>20</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>6</v>
+        <v>680</v>
       </c>
       <c r="D14" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">C14*D14</f>
-        <v>6</v>
+        <v>680</v>
       </c>
       <c r="G14" s="12"/>
     </row>
@@ -802,14 +810,17 @@
         <v>21</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>475</v>
+        <v>0</v>
       </c>
       <c r="D15" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">C15*D15</f>
-        <v>475</v>
+        <v>0</v>
+      </c>
+      <c r="F15" s="0" t="s">
+        <v>9</v>
       </c>
       <c r="G15" s="12"/>
     </row>
@@ -821,14 +832,14 @@
         <v>22</v>
       </c>
       <c r="C16" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" s="11" t="n">
         <v>2</v>
-      </c>
-      <c r="D16" s="11" t="n">
-        <v>1</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">C16*D16</f>
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G16" s="12"/>
     </row>
@@ -840,17 +851,14 @@
         <v>23</v>
       </c>
       <c r="C17" s="11" t="n">
-        <v>2</v>
+        <v>475</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">C17*D17</f>
-        <v>14</v>
-      </c>
-      <c r="F17" s="0" t="s">
-        <v>24</v>
+        <v>475</v>
       </c>
       <c r="G17" s="12"/>
     </row>
@@ -859,17 +867,17 @@
         <v>17</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" s="11" t="n">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="D18" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="12" t="n">
         <f aca="false">C18*D18</f>
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="G18" s="12"/>
     </row>
@@ -878,17 +886,20 @@
         <v>18</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19" s="11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E19" s="12" t="n">
         <f aca="false">C19*D19</f>
-        <v>5</v>
+        <v>14</v>
+      </c>
+      <c r="F19" s="0" t="s">
+        <v>26</v>
       </c>
       <c r="G19" s="12"/>
     </row>
@@ -900,14 +911,14 @@
         <v>27</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="D20" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">C20*D20</f>
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="G20" s="12"/>
     </row>
@@ -919,14 +930,14 @@
         <v>28</v>
       </c>
       <c r="C21" s="11" t="n">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D21" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">C21*D21</f>
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="G21" s="12"/>
     </row>
@@ -938,14 +949,14 @@
         <v>29</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D22" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">C22*D22</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G22" s="12"/>
     </row>
@@ -957,17 +968,14 @@
         <v>30</v>
       </c>
       <c r="C23" s="11" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D23" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">C23*D23</f>
-        <v>0</v>
-      </c>
-      <c r="F23" s="0" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="G23" s="12"/>
     </row>
@@ -979,10 +987,10 @@
         <v>31</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">C24*D24</f>
@@ -998,14 +1006,14 @@
         <v>32</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="12" t="n">
         <f aca="false">C25*D25</f>
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G25" s="12"/>
     </row>
@@ -1017,14 +1025,17 @@
         <v>33</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">C26*D26</f>
-        <v>25</v>
+        <v>0</v>
+      </c>
+      <c r="F26" s="0" t="s">
+        <v>9</v>
       </c>
       <c r="G26" s="12"/>
     </row>
@@ -1036,17 +1047,14 @@
         <v>34</v>
       </c>
       <c r="C27" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D27" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">C27*D27</f>
-        <v>0</v>
-      </c>
-      <c r="F27" s="0" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="G27" s="12"/>
     </row>
@@ -1058,17 +1066,14 @@
         <v>35</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">C28*D28</f>
-        <v>0</v>
-      </c>
-      <c r="F28" s="0" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G28" s="12"/>
     </row>
@@ -1080,17 +1085,14 @@
         <v>36</v>
       </c>
       <c r="C29" s="11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">C29*D29</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="0" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G29" s="12"/>
     </row>
@@ -1102,14 +1104,17 @@
         <v>37</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E30" s="12" t="n">
         <f aca="false">C30*D30</f>
-        <v>30</v>
+        <v>0</v>
+      </c>
+      <c r="F30" s="0" t="s">
+        <v>9</v>
       </c>
       <c r="G30" s="12"/>
     </row>
@@ -1121,14 +1126,17 @@
         <v>38</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E31" s="12" t="n">
         <f aca="false">C31*D31</f>
-        <v>24</v>
+        <v>0</v>
+      </c>
+      <c r="F31" s="0" t="s">
+        <v>9</v>
       </c>
       <c r="G31" s="12"/>
     </row>
@@ -1140,89 +1148,149 @@
         <v>39</v>
       </c>
       <c r="C32" s="11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">C32*D32</f>
-        <v>12</v>
+        <v>0</v>
+      </c>
+      <c r="F32" s="0" t="s">
+        <v>9</v>
       </c>
       <c r="G32" s="12"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="12"/>
+      <c r="A33" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <f aca="false">C33*D33</f>
+        <v>30</v>
+      </c>
       <c r="G33" s="12"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>40</v>
+      <c r="A34" s="4" t="n">
+        <v>33</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>41</v>
       </c>
       <c r="C34" s="11" t="n">
-        <v>70</v>
-      </c>
-      <c r="D34" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
+      </c>
+      <c r="D34" s="11" t="n">
+        <v>3</v>
       </c>
       <c r="E34" s="12" t="n">
         <f aca="false">C34*D34</f>
+        <v>24</v>
+      </c>
+      <c r="G34" s="12"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E35" s="12" t="n">
+        <f aca="false">C35*D35</f>
+        <v>18</v>
+      </c>
+      <c r="G35" s="12"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="12"/>
+      <c r="G36" s="12"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="12" t="n">
+        <f aca="false">C37*D37</f>
         <v>140</v>
       </c>
-      <c r="F34" s="13"/>
-      <c r="G34" s="14"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="14"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15"/>
-      <c r="B36" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="18" t="n">
+      <c r="F37" s="13"/>
+      <c r="G37" s="14"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="14"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15"/>
+      <c r="B39" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="18" t="n">
         <v>2000</v>
       </c>
-      <c r="F36" s="13"/>
-      <c r="G36" s="12"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4"/>
-      <c r="B37" s="19"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="12"/>
-    </row>
-    <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="1"/>
-      <c r="B38" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="24" t="n">
-        <f aca="false">SUM(E2:E37)</f>
-        <v>3803</v>
-      </c>
-      <c r="F38" s="25"/>
-      <c r="G38" s="21"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="12"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="12"/>
+    </row>
+    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1"/>
+      <c r="B41" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C41" s="23"/>
+      <c r="D41" s="23"/>
+      <c r="E41" s="24" t="n">
+        <f aca="false">SUM(E2:E40)</f>
+        <v>3885</v>
+      </c>
+      <c r="F41" s="25"/>
+      <c r="G41" s="21"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
removed stepper motor controller project to have its own repo
</commit_message>
<xml_diff>
--- a/rc_rover/BOM.xlsx
+++ b/rc_rover/BOM.xlsx
@@ -177,7 +177,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -200,14 +199,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -391,7 +388,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -444,11 +441,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -514,7 +515,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G41"/>
-  <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.39"/>
@@ -525,7 +526,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.5"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -585,7 +586,7 @@
         <f aca="false">C3*D3</f>
         <v>100</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="13" t="s">
         <v>9</v>
       </c>
       <c r="G3" s="12"/>
@@ -607,6 +608,7 @@
         <f aca="false">C4*D4</f>
         <v>10</v>
       </c>
+      <c r="F4" s="13"/>
       <c r="G4" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -625,7 +627,7 @@
       <c r="E5" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="13"/>
+      <c r="F5" s="11"/>
       <c r="G5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -645,7 +647,7 @@
         <f aca="false">C6*D6</f>
         <v>3</v>
       </c>
-      <c r="F6" s="13"/>
+      <c r="F6" s="11"/>
       <c r="G6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -665,7 +667,7 @@
         <f aca="false">C7*D7</f>
         <v>45</v>
       </c>
-      <c r="F7" s="13"/>
+      <c r="F7" s="11"/>
       <c r="G7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -685,7 +687,7 @@
         <f aca="false">C8*D8</f>
         <v>15</v>
       </c>
-      <c r="F8" s="13"/>
+      <c r="F8" s="11"/>
       <c r="G8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -705,6 +707,7 @@
         <f aca="false">C9*D9</f>
         <v>4</v>
       </c>
+      <c r="F9" s="13"/>
       <c r="G9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -724,6 +727,7 @@
         <f aca="false">C10*D10</f>
         <v>15</v>
       </c>
+      <c r="F10" s="13"/>
       <c r="G10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -743,6 +747,7 @@
         <f aca="false">C11*D11</f>
         <v>4</v>
       </c>
+      <c r="F11" s="13"/>
       <c r="G11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -762,6 +767,7 @@
         <f aca="false">C12*D12</f>
         <v>5</v>
       </c>
+      <c r="F12" s="13"/>
       <c r="G12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -781,6 +787,7 @@
         <f aca="false">C13*D13</f>
         <v>3</v>
       </c>
+      <c r="F13" s="13"/>
       <c r="G13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -800,6 +807,7 @@
         <f aca="false">C14*D14</f>
         <v>680</v>
       </c>
+      <c r="F14" s="13"/>
       <c r="G14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -819,7 +827,7 @@
         <f aca="false">C15*D15</f>
         <v>0</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="F15" s="13" t="s">
         <v>9</v>
       </c>
       <c r="G15" s="12"/>
@@ -841,6 +849,7 @@
         <f aca="false">C16*D16</f>
         <v>12</v>
       </c>
+      <c r="F16" s="13"/>
       <c r="G16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -860,6 +869,7 @@
         <f aca="false">C17*D17</f>
         <v>475</v>
       </c>
+      <c r="F17" s="13"/>
       <c r="G17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -879,6 +889,7 @@
         <f aca="false">C18*D18</f>
         <v>2</v>
       </c>
+      <c r="F18" s="13"/>
       <c r="G18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -898,7 +909,7 @@
         <f aca="false">C19*D19</f>
         <v>14</v>
       </c>
-      <c r="F19" s="0" t="s">
+      <c r="F19" s="13" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="12"/>
@@ -920,6 +931,7 @@
         <f aca="false">C20*D20</f>
         <v>30</v>
       </c>
+      <c r="F20" s="13"/>
       <c r="G20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -939,6 +951,7 @@
         <f aca="false">C21*D21</f>
         <v>45</v>
       </c>
+      <c r="F21" s="13"/>
       <c r="G21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -958,6 +971,7 @@
         <f aca="false">C22*D22</f>
         <v>5</v>
       </c>
+      <c r="F22" s="13"/>
       <c r="G22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -977,6 +991,7 @@
         <f aca="false">C23*D23</f>
         <v>12</v>
       </c>
+      <c r="F23" s="13"/>
       <c r="G23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -996,6 +1011,7 @@
         <f aca="false">C24*D24</f>
         <v>6</v>
       </c>
+      <c r="F24" s="13"/>
       <c r="G24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1015,6 +1031,7 @@
         <f aca="false">C25*D25</f>
         <v>1</v>
       </c>
+      <c r="F25" s="13"/>
       <c r="G25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1034,7 +1051,7 @@
         <f aca="false">C26*D26</f>
         <v>0</v>
       </c>
-      <c r="F26" s="0" t="s">
+      <c r="F26" s="13" t="s">
         <v>9</v>
       </c>
       <c r="G26" s="12"/>
@@ -1056,6 +1073,7 @@
         <f aca="false">C27*D27</f>
         <v>6</v>
       </c>
+      <c r="F27" s="13"/>
       <c r="G27" s="12"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1075,6 +1093,7 @@
         <f aca="false">C28*D28</f>
         <v>16</v>
       </c>
+      <c r="F28" s="13"/>
       <c r="G28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1094,6 +1113,7 @@
         <f aca="false">C29*D29</f>
         <v>25</v>
       </c>
+      <c r="F29" s="13"/>
       <c r="G29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1113,7 +1133,7 @@
         <f aca="false">C30*D30</f>
         <v>0</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="F30" s="13" t="s">
         <v>9</v>
       </c>
       <c r="G30" s="12"/>
@@ -1135,7 +1155,7 @@
         <f aca="false">C31*D31</f>
         <v>0</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="F31" s="13" t="s">
         <v>9</v>
       </c>
       <c r="G31" s="12"/>
@@ -1157,7 +1177,7 @@
         <f aca="false">C32*D32</f>
         <v>0</v>
       </c>
-      <c r="F32" s="0" t="s">
+      <c r="F32" s="13" t="s">
         <v>9</v>
       </c>
       <c r="G32" s="12"/>
@@ -1179,6 +1199,7 @@
         <f aca="false">C33*D33</f>
         <v>30</v>
       </c>
+      <c r="F33" s="13"/>
       <c r="G33" s="12"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1198,6 +1219,7 @@
         <f aca="false">C34*D34</f>
         <v>24</v>
       </c>
+      <c r="F34" s="13"/>
       <c r="G34" s="12"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1217,6 +1239,7 @@
         <f aca="false">C35*D35</f>
         <v>18</v>
       </c>
+      <c r="F35" s="13"/>
       <c r="G35" s="12"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1225,6 +1248,7 @@
       <c r="C36" s="11"/>
       <c r="D36" s="11"/>
       <c r="E36" s="12"/>
+      <c r="F36" s="13"/>
       <c r="G36" s="12"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1244,7 +1268,7 @@
         <f aca="false">C37*D37</f>
         <v>140</v>
       </c>
-      <c r="F37" s="13"/>
+      <c r="F37" s="11"/>
       <c r="G37" s="14"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1253,44 +1277,44 @@
       <c r="C38" s="11"/>
       <c r="D38" s="4"/>
       <c r="E38" s="12"/>
-      <c r="F38" s="13"/>
+      <c r="F38" s="15"/>
       <c r="G38" s="14"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15"/>
-      <c r="B39" s="16" t="s">
+      <c r="A39" s="16"/>
+      <c r="B39" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="18" t="n">
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="19" t="n">
         <v>2000</v>
       </c>
-      <c r="F39" s="13"/>
+      <c r="F39" s="15"/>
       <c r="G39" s="12"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4"/>
-      <c r="B40" s="19"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="13"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="15"/>
       <c r="G40" s="12"/>
     </row>
-    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1"/>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C41" s="23"/>
-      <c r="D41" s="23"/>
-      <c r="E41" s="24" t="n">
+      <c r="C41" s="24"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="25" t="n">
         <f aca="false">SUM(E2:E40)</f>
         <v>3885</v>
       </c>
-      <c r="F41" s="25"/>
-      <c r="G41" s="21"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="22"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>